<commit_message>
🤖 Atualização Automática: Dados IPMA (Minuto 15)
</commit_message>
<xml_diff>
--- a/Painel_Mestre_IPMA.xlsx
+++ b/Painel_Mestre_IPMA.xlsx
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25.8</v>
+        <v>17.6</v>
       </c>
       <c r="C2" t="n">
-        <v>12.4</v>
+        <v>13.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.948</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.498</v>
+        <v>0.847</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -531,30 +531,30 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24.9</v>
+        <v>17</v>
       </c>
       <c r="C3" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.914</v>
+        <v>0.995</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5429999999999999</v>
+        <v>0.862</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -575,16 +575,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>18.3</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9359999999999999</v>
+        <v>0.985</v>
       </c>
       <c r="E4" t="n">
-        <v>0.474</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -619,16 +619,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>18.6</v>
       </c>
       <c r="C5" t="n">
-        <v>14.7</v>
+        <v>13.5</v>
       </c>
       <c r="D5" t="n">
-        <v>0.852</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0.517</v>
+        <v>0.773</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -637,12 +637,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva forte</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -663,16 +663,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>15.5</v>
       </c>
       <c r="C6" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.914</v>
+        <v>0.982</v>
       </c>
       <c r="E6" t="n">
-        <v>0.49</v>
+        <v>0.861</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25.9</v>
+        <v>17.7</v>
       </c>
       <c r="C7" t="n">
-        <v>12.6</v>
+        <v>13.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.948</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5</v>
+        <v>0.848</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -751,16 +751,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26.5</v>
+        <v>17.4</v>
       </c>
       <c r="C8" t="n">
-        <v>12.4</v>
+        <v>13.2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.508</v>
+        <v>0.85</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -795,16 +795,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>26.6</v>
+        <v>18.3</v>
       </c>
       <c r="C9" t="n">
-        <v>13.1</v>
+        <v>13.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.945</v>
+        <v>0.98</v>
       </c>
       <c r="E9" t="n">
-        <v>0.488</v>
+        <v>0.8370000000000001</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25.5</v>
+        <v>16.9</v>
       </c>
       <c r="C10" t="n">
-        <v>14.8</v>
+        <v>13.6</v>
       </c>
       <c r="D10" t="n">
-        <v>0.986</v>
+        <v>0.9990000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.583</v>
+        <v>0.848</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -883,16 +883,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>27.4</v>
+        <v>17.9</v>
       </c>
       <c r="C11" t="n">
-        <v>12.2</v>
+        <v>11.7</v>
       </c>
       <c r="D11" t="n">
-        <v>0.965</v>
+        <v>0.9890000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.509</v>
+        <v>0.872</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -927,16 +927,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>18</v>
+        <v>20.2</v>
       </c>
       <c r="C12" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0.9940000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.843</v>
+        <v>0.677</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -945,12 +945,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -971,16 +971,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>17.5</v>
+        <v>18.6</v>
       </c>
       <c r="C13" t="n">
-        <v>13.5</v>
+        <v>13.1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.995</v>
+        <v>0.9740000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>0.856</v>
+        <v>0.736</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1015,16 +1015,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19</v>
+        <v>21.3</v>
       </c>
       <c r="C14" t="n">
-        <v>12.8</v>
+        <v>12.2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.995</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>0.78</v>
+        <v>0.5760000000000001</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1059,16 +1059,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19.6</v>
+        <v>21.7</v>
       </c>
       <c r="C15" t="n">
         <v>13.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.995</v>
+        <v>0.9209999999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.779</v>
+        <v>0.574</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16.3</v>
+        <v>17.9</v>
       </c>
       <c r="C16" t="n">
-        <v>12.2</v>
+        <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>0.992</v>
+        <v>0.973</v>
       </c>
       <c r="E16" t="n">
-        <v>0.846</v>
+        <v>0.6729999999999999</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1147,16 +1147,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>18.1</v>
+        <v>20.4</v>
       </c>
       <c r="C17" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="E17" t="n">
-        <v>0.845</v>
+        <v>0.6779999999999999</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1191,16 +1191,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18.3</v>
+        <v>19.7</v>
       </c>
       <c r="C18" t="n">
-        <v>12.6</v>
+        <v>12.2</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0.985</v>
       </c>
       <c r="E18" t="n">
-        <v>0.856</v>
+        <v>0.7090000000000001</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1235,16 +1235,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18.6</v>
+        <v>20.7</v>
       </c>
       <c r="C19" t="n">
-        <v>13.7</v>
+        <v>12.8</v>
       </c>
       <c r="D19" t="n">
-        <v>0.995</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>0.838</v>
+        <v>0.665</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1253,12 +1253,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1279,16 +1279,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17.6</v>
+        <v>18.3</v>
       </c>
       <c r="C20" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>0.997</v>
       </c>
       <c r="E20" t="n">
-        <v>0.799</v>
+        <v>0.7190000000000001</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1323,16 +1323,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>18.3</v>
+        <v>20.2</v>
       </c>
       <c r="C21" t="n">
-        <v>11.9</v>
+        <v>10.8</v>
       </c>
       <c r="D21" t="n">
-        <v>0.991</v>
+        <v>0.971</v>
       </c>
       <c r="E21" t="n">
-        <v>0.856</v>
+        <v>0.713</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1341,12 +1341,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1367,16 +1367,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>20.1</v>
+        <v>21.8</v>
       </c>
       <c r="C22" t="n">
-        <v>12.2</v>
+        <v>9.4</v>
       </c>
       <c r="D22" t="n">
-        <v>0.991</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.65</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1411,30 +1411,30 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="C23" t="n">
-        <v>12.9</v>
+        <v>11.6</v>
       </c>
       <c r="D23" t="n">
-        <v>0.975</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>0.736</v>
+        <v>0.774</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1455,16 +1455,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.98</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5720000000000001</v>
+        <v>0.679</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1499,16 +1499,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>22.6</v>
+        <v>23.1</v>
       </c>
       <c r="C25" t="n">
-        <v>13</v>
+        <v>10.8</v>
       </c>
       <c r="D25" t="n">
-        <v>0.898</v>
+        <v>0.929</v>
       </c>
       <c r="E25" t="n">
-        <v>0.5579999999999999</v>
+        <v>0.6409999999999999</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1543,16 +1543,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>17.7</v>
+        <v>19</v>
       </c>
       <c r="C26" t="n">
-        <v>10.4</v>
+        <v>9.1</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9790000000000001</v>
+        <v>0.993</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6579999999999999</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1587,16 +1587,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>20.2</v>
+        <v>21.9</v>
       </c>
       <c r="C27" t="n">
-        <v>12.3</v>
+        <v>9.5</v>
       </c>
       <c r="D27" t="n">
-        <v>0.991</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.655</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1631,16 +1631,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>19.7</v>
+        <v>21.1</v>
       </c>
       <c r="C28" t="n">
-        <v>11.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D28" t="n">
-        <v>0.998</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6709999999999999</v>
+        <v>0.662</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1675,16 +1675,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="C29" t="n">
-        <v>12.2</v>
+        <v>11.1</v>
       </c>
       <c r="D29" t="n">
-        <v>0.946</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.675</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1719,16 +1719,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="C30" t="n">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="D30" t="n">
-        <v>0.983</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>0.705</v>
+        <v>0.778</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1766,27 +1766,27 @@
         <v>20.5</v>
       </c>
       <c r="C31" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D31" t="n">
-        <v>0.9670000000000001</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>0.725</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>22.4</v>
+        <v>19.2</v>
       </c>
       <c r="C32" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="D32" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>0.615</v>
+        <v>0.743</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1825,12 +1825,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1851,16 +1851,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>18.9</v>
+        <v>18.1</v>
       </c>
       <c r="C33" t="n">
-        <v>11.4</v>
+        <v>12.2</v>
       </c>
       <c r="D33" t="n">
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>0.7509999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1869,12 +1869,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1895,16 +1895,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>22.6</v>
+        <v>19.6</v>
       </c>
       <c r="C34" t="n">
-        <v>10.3</v>
+        <v>10.9</v>
       </c>
       <c r="D34" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>0.58</v>
+        <v>0.675</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1939,16 +1939,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C35" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="D35" t="n">
-        <v>0.9359999999999999</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>0.599</v>
+        <v>0.643</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1983,16 +1983,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>19.6</v>
+        <v>17.2</v>
       </c>
       <c r="C36" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D36" t="n">
-        <v>0.9470000000000001</v>
+        <v>0.987</v>
       </c>
       <c r="E36" t="n">
-        <v>0.638</v>
+        <v>0.6940000000000001</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2027,16 +2027,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>22.5</v>
+        <v>19.3</v>
       </c>
       <c r="C37" t="n">
-        <v>9.9</v>
+        <v>10.9</v>
       </c>
       <c r="D37" t="n">
-        <v>0.987</v>
+        <v>0.993</v>
       </c>
       <c r="E37" t="n">
-        <v>0.615</v>
+        <v>0.748</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2045,12 +2045,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2071,16 +2071,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>21.5</v>
+        <v>19</v>
       </c>
       <c r="C38" t="n">
-        <v>9.199999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>0.635</v>
+        <v>0.748</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2089,12 +2089,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2115,16 +2115,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>22.2</v>
+        <v>20.1</v>
       </c>
       <c r="C39" t="n">
-        <v>10.5</v>
+        <v>11.4</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>0.626</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2159,16 +2159,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>18.3</v>
+        <v>17.4</v>
       </c>
       <c r="C40" t="n">
-        <v>10.3</v>
+        <v>10.7</v>
       </c>
       <c r="D40" t="n">
-        <v>0.9990000000000001</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>0.762</v>
+        <v>0.7979999999999999</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2177,12 +2177,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2203,16 +2203,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>21.1</v>
+        <v>19.6</v>
       </c>
       <c r="C41" t="n">
-        <v>9.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>0.701</v>
+        <v>0.7090000000000001</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -2247,16 +2247,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>18.5</v>
+        <v>19.7</v>
       </c>
       <c r="C42" t="n">
-        <v>10.9</v>
+        <v>9.4</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0.985</v>
       </c>
       <c r="E42" t="n">
-        <v>0.7909999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2265,12 +2265,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2291,25 +2291,25 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="C43" t="n">
-        <v>11.7</v>
+        <v>11</v>
       </c>
       <c r="D43" t="n">
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>0.768</v>
+        <v>0.728</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2335,16 +2335,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="C44" t="n">
-        <v>10.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>0.9890000000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.608</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2379,16 +2379,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="C45" t="n">
-        <v>11.7</v>
+        <v>10.4</v>
       </c>
       <c r="D45" t="n">
-        <v>0.98</v>
+        <v>0.9790000000000001</v>
       </c>
       <c r="E45" t="n">
-        <v>0.6509999999999999</v>
+        <v>0.593</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2397,12 +2397,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2423,16 +2423,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>16.3</v>
+        <v>17</v>
       </c>
       <c r="C46" t="n">
-        <v>9.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>0.9990000000000001</v>
       </c>
       <c r="E46" t="n">
-        <v>0.7859999999999999</v>
+        <v>0.6409999999999999</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2467,16 +2467,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>18.7</v>
+        <v>19.8</v>
       </c>
       <c r="C47" t="n">
-        <v>11.1</v>
+        <v>9.5</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="E47" t="n">
-        <v>0.792</v>
+        <v>0.604</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2511,16 +2511,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="C48" t="n">
-        <v>10.5</v>
+        <v>9.1</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>0.787</v>
+        <v>0.637</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2529,12 +2529,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2555,16 +2555,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="C49" t="n">
-        <v>11.2</v>
+        <v>10.1</v>
       </c>
       <c r="D49" t="n">
         <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>0.772</v>
+        <v>0.634</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16.9</v>
+        <v>17.4</v>
       </c>
       <c r="C50" t="n">
-        <v>10.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D50" t="n">
         <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>0.78</v>
+        <v>0.74</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2643,16 +2643,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>19.2</v>
+        <v>19</v>
       </c>
       <c r="C51" t="n">
-        <v>10</v>
+        <v>8.6</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>0.74</v>
+        <v>0.653</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2687,16 +2687,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>18.6</v>
+        <v>19.9</v>
       </c>
       <c r="C52" t="n">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>0.605</v>
+        <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2731,16 +2731,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>17.4</v>
+        <v>17.7</v>
       </c>
       <c r="C53" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="D53" t="n">
-        <v>0.902</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>0.6679999999999999</v>
+        <v>0</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2775,16 +2775,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>18.8</v>
+        <v>19.6</v>
       </c>
       <c r="C54" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2793,12 +2793,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2819,16 +2819,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>20</v>
+        <v>20.6</v>
       </c>
       <c r="C55" t="n">
-        <v>10.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0.5710000000000001</v>
+        <v>0</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2863,16 +2863,16 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>16.2</v>
+        <v>17.4</v>
       </c>
       <c r="C56" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>0.634</v>
+        <v>0</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2881,12 +2881,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2907,16 +2907,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>18.7</v>
+        <v>20.1</v>
       </c>
       <c r="C57" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2951,16 +2951,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>18.6</v>
+        <v>19.6</v>
       </c>
       <c r="C58" t="n">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>0.598</v>
+        <v>0</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2995,16 +2995,16 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>19</v>
+        <v>20.1</v>
       </c>
       <c r="C59" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="D59" t="n">
-        <v>0.987</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>0.617</v>
+        <v>0</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -3039,20 +3039,20 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17.5</v>
+        <v>17.8</v>
       </c>
       <c r="C60" t="n">
-        <v>9.9</v>
+        <v>9.1</v>
       </c>
       <c r="D60" t="n">
-        <v>0.982</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>0.65</v>
+        <v>0</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -3083,16 +3083,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>18.8</v>
+        <v>19.5</v>
       </c>
       <c r="C61" t="n">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>0.618</v>
+        <v>0</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>18.9</v>
+        <v>21.9</v>
       </c>
       <c r="C62" t="n">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -3145,12 +3145,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3171,10 +3171,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>17.8</v>
+        <v>19.2</v>
       </c>
       <c r="C63" t="n">
-        <v>10.3</v>
+        <v>10.5</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3215,10 +3215,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>19.2</v>
+        <v>21.6</v>
       </c>
       <c r="C64" t="n">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -3233,12 +3233,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>20.5</v>
+        <v>22.6</v>
       </c>
       <c r="C65" t="n">
         <v>9.699999999999999</v>
@@ -3277,12 +3277,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3303,10 +3303,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>16.8</v>
+        <v>19.5</v>
       </c>
       <c r="C66" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -3321,12 +3321,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3347,10 +3347,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C67" t="n">
-        <v>8.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -3365,12 +3365,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3391,10 +3391,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>19</v>
+        <v>21.6</v>
       </c>
       <c r="C68" t="n">
-        <v>7.9</v>
+        <v>8.5</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -3409,12 +3409,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3435,10 +3435,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>19.6</v>
+        <v>22.1</v>
       </c>
       <c r="C69" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -3453,12 +3453,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>17.8</v>
+        <v>19.8</v>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3523,10 +3523,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>19.4</v>
+        <v>21.4</v>
       </c>
       <c r="C71" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -3541,12 +3541,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3567,10 +3567,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>20.1</v>
+        <v>22.2</v>
       </c>
       <c r="C72" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -3585,12 +3585,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3611,10 +3611,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>18.7</v>
+        <v>19.6</v>
       </c>
       <c r="C73" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3655,10 +3655,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>20.1</v>
+        <v>21.8</v>
       </c>
       <c r="C74" t="n">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3699,10 +3699,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>21.3</v>
+        <v>22.8</v>
       </c>
       <c r="C75" t="n">
-        <v>9.5</v>
+        <v>10.8</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3743,10 +3743,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>17.9</v>
+        <v>19.7</v>
       </c>
       <c r="C76" t="n">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3787,10 +3787,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>20.2</v>
+        <v>22.3</v>
       </c>
       <c r="C77" t="n">
-        <v>8.9</v>
+        <v>10.5</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -3805,12 +3805,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3831,10 +3831,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>20.2</v>
+        <v>21.9</v>
       </c>
       <c r="C78" t="n">
-        <v>7.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3875,10 +3875,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>20.5</v>
+        <v>22.3</v>
       </c>
       <c r="C79" t="n">
-        <v>8.9</v>
+        <v>10.2</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -3893,12 +3893,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3919,10 +3919,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>19</v>
+        <v>20.2</v>
       </c>
       <c r="C80" t="n">
-        <v>8.699999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3963,10 +3963,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>20.5</v>
+        <v>21.8</v>
       </c>
       <c r="C81" t="n">
-        <v>7.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -4007,10 +4007,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>21.6</v>
+        <v>21.2</v>
       </c>
       <c r="C82" t="n">
-        <v>8.9</v>
+        <v>10.4</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4051,10 +4051,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>19.7</v>
+        <v>19</v>
       </c>
       <c r="C83" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -4069,12 +4069,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4095,10 +4095,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="C84" t="n">
-        <v>8.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4139,10 +4139,10 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>22.8</v>
+        <v>22.1</v>
       </c>
       <c r="C85" t="n">
-        <v>9.6</v>
+        <v>10.9</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -4157,12 +4157,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4183,10 +4183,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>19.4</v>
+        <v>18.9</v>
       </c>
       <c r="C86" t="n">
-        <v>7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4227,10 +4227,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>21.7</v>
+        <v>21.4</v>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>10.6</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4271,10 +4271,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>21.8</v>
+        <v>21</v>
       </c>
       <c r="C88" t="n">
-        <v>7.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D88" t="n">
         <v>0</v>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4315,10 +4315,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>22</v>
+        <v>21.6</v>
       </c>
       <c r="C89" t="n">
-        <v>8.699999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -4333,12 +4333,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4359,10 +4359,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>20.6</v>
+        <v>19.2</v>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4403,10 +4403,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>21.9</v>
+        <v>21</v>
       </c>
       <c r="C91" t="n">
-        <v>7.4</v>
+        <v>9.1</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -4421,12 +4421,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Atualização Automática: XLSX e CSV
</commit_message>
<xml_diff>
--- a/Painel_Mestre_IPMA.xlsx
+++ b/Painel_Mestre_IPMA.xlsx
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19.1</v>
+        <v>19.6</v>
       </c>
       <c r="C2" t="n">
-        <v>12.9</v>
+        <v>12.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.993</v>
+        <v>0.998</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8170000000000001</v>
+        <v>0.7070000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -505,12 +505,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -531,16 +531,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="C3" t="n">
-        <v>13.5</v>
+        <v>12.8</v>
       </c>
       <c r="D3" t="n">
-        <v>0.995</v>
+        <v>0.96</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8390000000000001</v>
+        <v>0.743</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -549,12 +549,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -575,16 +575,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18.7</v>
+        <v>20.3</v>
       </c>
       <c r="C4" t="n">
-        <v>12.8</v>
+        <v>12.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9690000000000001</v>
+        <v>0.968</v>
       </c>
       <c r="E4" t="n">
-        <v>0.825</v>
+        <v>0.6459999999999999</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -619,16 +619,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19.8</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="D5" t="n">
-        <v>0.981</v>
+        <v>0.9690000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7809999999999999</v>
+        <v>0.632</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -663,16 +663,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17.2</v>
+        <v>18.1</v>
       </c>
       <c r="C6" t="n">
-        <v>12.1</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>0.997</v>
+        <v>0.992</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.647</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -681,12 +681,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19.2</v>
+        <v>19.7</v>
       </c>
       <c r="C7" t="n">
-        <v>13.1</v>
+        <v>12.2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.992</v>
+        <v>0.998</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.7090000000000001</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,12 +725,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -751,16 +751,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18.8</v>
+        <v>20</v>
       </c>
       <c r="C8" t="n">
-        <v>12.9</v>
+        <v>11.1</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8190000000000001</v>
+        <v>0.642</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -774,7 +774,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -795,20 +795,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>20.8</v>
       </c>
       <c r="C9" t="n">
-        <v>13.5</v>
+        <v>11.8</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9940000000000001</v>
+        <v>0.971</v>
       </c>
       <c r="E9" t="n">
-        <v>0.821</v>
+        <v>0.645</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="C10" t="n">
-        <v>13.4</v>
+        <v>11.4</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="E10" t="n">
-        <v>0.787</v>
+        <v>0.675</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -857,12 +857,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Chuva forte</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -883,20 +883,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19.3</v>
+        <v>20.3</v>
       </c>
       <c r="C11" t="n">
-        <v>11.9</v>
+        <v>10.1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.981</v>
+        <v>0.973</v>
       </c>
       <c r="E11" t="n">
-        <v>0.847</v>
+        <v>0.701</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Chuva moderada</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -927,16 +927,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20.4</v>
+        <v>20.7</v>
       </c>
       <c r="C12" t="n">
-        <v>12.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9990000000000001</v>
+        <v>0.9940000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6809999999999999</v>
+        <v>0.6509999999999999</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -974,27 +974,27 @@
         <v>18.4</v>
       </c>
       <c r="C13" t="n">
-        <v>13.1</v>
+        <v>11</v>
       </c>
       <c r="D13" t="n">
-        <v>0.963</v>
+        <v>0.996</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7659999999999999</v>
+        <v>0.7559999999999999</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1015,16 +1015,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>22.1</v>
+        <v>19.9</v>
       </c>
       <c r="C14" t="n">
-        <v>12.3</v>
+        <v>9.9</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9259999999999999</v>
+        <v>0.953</v>
       </c>
       <c r="E14" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.659</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1059,30 +1059,30 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22.7</v>
+        <v>21.4</v>
       </c>
       <c r="C15" t="n">
-        <v>13.2</v>
+        <v>10.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.894</v>
+        <v>0.946</v>
       </c>
       <c r="E15" t="n">
-        <v>0.5479999999999999</v>
+        <v>0.636</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17.7</v>
+        <v>18.1</v>
       </c>
       <c r="C16" t="n">
-        <v>10.5</v>
+        <v>8.1</v>
       </c>
       <c r="D16" t="n">
-        <v>0.983</v>
+        <v>0.9840000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7190000000000001</v>
+        <v>0.674</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1121,12 +1121,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1147,16 +1147,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="C17" t="n">
-        <v>12.4</v>
+        <v>9.4</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9990000000000001</v>
+        <v>0.993</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6829999999999999</v>
+        <v>0.653</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1191,16 +1191,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>19.5</v>
+        <v>20.3</v>
       </c>
       <c r="C18" t="n">
-        <v>11.3</v>
+        <v>9.6</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7070000000000001</v>
+        <v>0.642</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1238,27 +1238,27 @@
         <v>20.7</v>
       </c>
       <c r="C19" t="n">
-        <v>12.3</v>
+        <v>9.9</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9590000000000001</v>
+        <v>0.998</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6920000000000001</v>
+        <v>0.6659999999999999</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1279,16 +1279,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>18.7</v>
+        <v>17.5</v>
       </c>
       <c r="C20" t="n">
-        <v>11.8</v>
+        <v>10.2</v>
       </c>
       <c r="D20" t="n">
-        <v>0.997</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>0.72</v>
+        <v>0.7390000000000001</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1297,12 +1297,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1323,30 +1323,30 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>20.2</v>
+        <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>0.983</v>
+        <v>0.996</v>
       </c>
       <c r="E21" t="n">
-        <v>0.7490000000000001</v>
+        <v>0.711</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1367,16 +1367,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>20.8</v>
+        <v>19.2</v>
       </c>
       <c r="C22" t="n">
-        <v>10</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>0.665</v>
+        <v>0.6659999999999999</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1411,16 +1411,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18.4</v>
+        <v>17.6</v>
       </c>
       <c r="C23" t="n">
-        <v>12.3</v>
+        <v>10.2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.988</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>0.758</v>
+        <v>0.787</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1455,16 +1455,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>21.1</v>
+        <v>19.1</v>
       </c>
       <c r="C24" t="n">
-        <v>10.1</v>
+        <v>9.5</v>
       </c>
       <c r="D24" t="n">
-        <v>0.983</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6509999999999999</v>
+        <v>0.644</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1499,16 +1499,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>22.2</v>
+        <v>20.3</v>
       </c>
       <c r="C25" t="n">
-        <v>10.9</v>
+        <v>10.2</v>
       </c>
       <c r="D25" t="n">
-        <v>0.958</v>
+        <v>0.9670000000000001</v>
       </c>
       <c r="E25" t="n">
-        <v>0.628</v>
+        <v>0.629</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1543,16 +1543,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>18.1</v>
+        <v>16.6</v>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>7.7</v>
       </c>
       <c r="D26" t="n">
-        <v>0.992</v>
+        <v>0.993</v>
       </c>
       <c r="E26" t="n">
-        <v>0.695</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1587,16 +1587,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>20.9</v>
+        <v>19.3</v>
       </c>
       <c r="C27" t="n">
-        <v>10.2</v>
+        <v>9.4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>0.665</v>
+        <v>0.6659999999999999</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1631,16 +1631,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="C28" t="n">
-        <v>10.7</v>
+        <v>8.5</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6970000000000001</v>
+        <v>0.7240000000000001</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1675,16 +1675,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>21</v>
+        <v>19.7</v>
       </c>
       <c r="C29" t="n">
-        <v>10.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D29" t="n">
-        <v>0.9940000000000001</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6859999999999999</v>
+        <v>0.672</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1719,16 +1719,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>17.5</v>
+        <v>16.6</v>
       </c>
       <c r="C30" t="n">
-        <v>11.3</v>
+        <v>8.5</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0.996</v>
       </c>
       <c r="E30" t="n">
-        <v>0.784</v>
+        <v>0.7879999999999999</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1763,16 +1763,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>20.3</v>
+        <v>19.2</v>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>8.4</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7170000000000001</v>
+        <v>0.698</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -1807,16 +1807,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>19.5</v>
+        <v>17.8</v>
       </c>
       <c r="C32" t="n">
-        <v>10.6</v>
+        <v>9.1</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="E32" t="n">
-        <v>0.645</v>
+        <v>0.726</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -1851,16 +1851,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>17.9</v>
+        <v>16.8</v>
       </c>
       <c r="C33" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E33" t="n">
-        <v>0.747</v>
+        <v>0.73</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -1895,16 +1895,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>19.6</v>
+        <v>16.6</v>
       </c>
       <c r="C34" t="n">
-        <v>10.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E34" t="n">
-        <v>0.648</v>
+        <v>0.795</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -1939,16 +1939,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>21.2</v>
+        <v>18</v>
       </c>
       <c r="C35" t="n">
-        <v>11.4</v>
+        <v>10.1</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>0.929</v>
       </c>
       <c r="E35" t="n">
-        <v>0.633</v>
+        <v>0.721</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -1983,16 +1983,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>17.7</v>
+        <v>16</v>
       </c>
       <c r="C36" t="n">
-        <v>8.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="E36" t="n">
-        <v>0.633</v>
+        <v>0.721</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2027,16 +2027,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>19.6</v>
+        <v>17.9</v>
       </c>
       <c r="C37" t="n">
-        <v>10.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="E37" t="n">
-        <v>0.65</v>
+        <v>0.731</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2071,16 +2071,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>19.4</v>
+        <v>18.7</v>
       </c>
       <c r="C38" t="n">
-        <v>9.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.7120000000000001</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2115,16 +2115,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20.4</v>
+        <v>18.3</v>
       </c>
       <c r="C39" t="n">
-        <v>10.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>0.622</v>
+        <v>0.703</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2159,16 +2159,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>17.9</v>
+        <v>17.2</v>
       </c>
       <c r="C40" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
-        <v>0.988</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>0.769</v>
+        <v>0.758</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2203,16 +2203,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>19.9</v>
+        <v>18.2</v>
       </c>
       <c r="C41" t="n">
-        <v>9.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>0.664</v>
+        <v>0.6920000000000001</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -2247,16 +2247,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>18.6</v>
+        <v>17.8</v>
       </c>
       <c r="C42" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0.9620000000000001</v>
       </c>
       <c r="E42" t="n">
-        <v>0.599</v>
+        <v>0.597</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2291,20 +2291,20 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>16.5</v>
+        <v>16.6</v>
       </c>
       <c r="C43" t="n">
-        <v>10.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D43" t="n">
-        <v>0.977</v>
+        <v>0.9109999999999999</v>
       </c>
       <c r="E43" t="n">
-        <v>0.647</v>
+        <v>0.631</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2335,16 +2335,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="C44" t="n">
-        <v>8.5</v>
+        <v>8.1</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E44" t="n">
-        <v>0.6679999999999999</v>
+        <v>0.657</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2382,13 +2382,13 @@
         <v>18.5</v>
       </c>
       <c r="C45" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D45" t="n">
-        <v>0.9670000000000001</v>
+        <v>0.903</v>
       </c>
       <c r="E45" t="n">
-        <v>0.619</v>
+        <v>0.599</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2423,16 +2423,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>16</v>
+        <v>15.5</v>
       </c>
       <c r="C46" t="n">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="D46" t="n">
-        <v>0.992</v>
+        <v>0.96</v>
       </c>
       <c r="E46" t="n">
-        <v>0.628</v>
+        <v>0.614</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2467,16 +2467,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>18.8</v>
+        <v>17.9</v>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>8.1</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0.963</v>
       </c>
       <c r="E47" t="n">
-        <v>0.595</v>
+        <v>0.602</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2511,16 +2511,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>18.4</v>
+        <v>17.8</v>
       </c>
       <c r="C48" t="n">
-        <v>8.4</v>
+        <v>7.3</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>0.598</v>
+        <v>0.607</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2555,16 +2555,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="C49" t="n">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>0.973</v>
       </c>
       <c r="E49" t="n">
-        <v>0.606</v>
+        <v>0.625</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2599,16 +2599,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16.9</v>
+        <v>16.2</v>
       </c>
       <c r="C50" t="n">
-        <v>9.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="D50" t="n">
-        <v>0.961</v>
+        <v>0.9840000000000001</v>
       </c>
       <c r="E50" t="n">
-        <v>0.6709999999999999</v>
+        <v>0.628</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2643,25 +2643,25 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>18.3</v>
+        <v>17.9</v>
       </c>
       <c r="C51" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>0.579</v>
+        <v>0.62</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -2687,16 +2687,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="C52" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="D52" t="n">
-        <v>0.924</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2731,16 +2731,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>16.5</v>
+        <v>17.8</v>
       </c>
       <c r="C53" t="n">
-        <v>10.2</v>
+        <v>9.6</v>
       </c>
       <c r="D53" t="n">
-        <v>0.8390000000000001</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>0.601</v>
+        <v>0</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2775,16 +2775,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="C54" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="D54" t="n">
-        <v>0.9209999999999999</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>0.5379999999999999</v>
+        <v>0</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2793,7 +2793,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2819,16 +2819,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>19.5</v>
+        <v>20.1</v>
       </c>
       <c r="C55" t="n">
-        <v>9.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D55" t="n">
-        <v>0.8640000000000001</v>
+        <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0.493</v>
+        <v>0</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2863,16 +2863,16 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>16.1</v>
+        <v>17.2</v>
       </c>
       <c r="C56" t="n">
-        <v>6.9</v>
+        <v>6.1</v>
       </c>
       <c r="D56" t="n">
-        <v>0.892</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>0.5529999999999999</v>
+        <v>0</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2907,16 +2907,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="C57" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="D57" t="n">
-        <v>0.919</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>0.524</v>
+        <v>0</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2951,16 +2951,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>17.9</v>
+        <v>19.7</v>
       </c>
       <c r="C58" t="n">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="D58" t="n">
-        <v>0.958</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5529999999999999</v>
+        <v>0</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -2995,16 +2995,16 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="C59" t="n">
-        <v>8.699999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="D59" t="n">
-        <v>0.945</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>0.5329999999999999</v>
+        <v>0</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3039,20 +3039,20 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17</v>
+        <v>17.8</v>
       </c>
       <c r="C60" t="n">
-        <v>8.699999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="D60" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>0.597</v>
+        <v>0</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Sem chuva</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3083,16 +3083,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>18.5</v>
+        <v>19.5</v>
       </c>
       <c r="C61" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>0.537</v>
+        <v>0</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>20.9</v>
+        <v>21.8</v>
       </c>
       <c r="C62" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3171,10 +3171,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>18.1</v>
+        <v>19.3</v>
       </c>
       <c r="C63" t="n">
-        <v>10.1</v>
+        <v>9.1</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -3189,7 +3189,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3215,10 +3215,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>19.7</v>
+        <v>20.5</v>
       </c>
       <c r="C64" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3259,10 +3259,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>21.3</v>
+        <v>22.1</v>
       </c>
       <c r="C65" t="n">
-        <v>8.800000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3303,10 +3303,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>18.1</v>
+        <v>19.3</v>
       </c>
       <c r="C66" t="n">
-        <v>6.6</v>
+        <v>5.5</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3347,10 +3347,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>21</v>
+        <v>21.9</v>
       </c>
       <c r="C67" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3391,10 +3391,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>20.2</v>
+        <v>21.8</v>
       </c>
       <c r="C68" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3435,10 +3435,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>20.8</v>
+        <v>21.9</v>
       </c>
       <c r="C69" t="n">
-        <v>8.300000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>19.2</v>
+        <v>19.9</v>
       </c>
       <c r="C70" t="n">
-        <v>8.5</v>
+        <v>7.7</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3523,10 +3523,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>20.3</v>
+        <v>21.6</v>
       </c>
       <c r="C71" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>22.6</v>
+        <v>21.9</v>
       </c>
       <c r="C72" t="n">
         <v>8.300000000000001</v>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3611,10 +3611,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="C73" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3655,10 +3655,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>21.7</v>
+        <v>21.1</v>
       </c>
       <c r="C74" t="n">
-        <v>8.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -3673,12 +3673,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3699,10 +3699,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="C75" t="n">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
@@ -3717,12 +3717,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3743,10 +3743,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>20.1</v>
+        <v>19.8</v>
       </c>
       <c r="C76" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -3761,12 +3761,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3787,10 +3787,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>22.7</v>
+        <v>22</v>
       </c>
       <c r="C77" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3831,10 +3831,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="C78" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3875,10 +3875,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>22.8</v>
+        <v>22.3</v>
       </c>
       <c r="C79" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3919,10 +3919,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C80" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3963,10 +3963,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>22.4</v>
+        <v>22</v>
       </c>
       <c r="C81" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4007,10 +4007,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>22.3</v>
+        <v>21.1</v>
       </c>
       <c r="C82" t="n">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>19</v>
+        <v>18.7</v>
       </c>
       <c r="C83" t="n">
         <v>10.7</v>
@@ -4069,12 +4069,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4095,10 +4095,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>21.9</v>
+        <v>20.7</v>
       </c>
       <c r="C84" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -4113,12 +4113,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Chuva fraca</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>23.2</v>
+        <v>22</v>
       </c>
       <c r="C85" t="n">
         <v>9.800000000000001</v>
@@ -4157,12 +4157,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4183,10 +4183,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C86" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -4201,12 +4201,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4227,10 +4227,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>22.4</v>
+        <v>21.2</v>
       </c>
       <c r="C87" t="n">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4271,10 +4271,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>21.8</v>
+        <v>21.2</v>
       </c>
       <c r="C88" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D88" t="n">
         <v>0</v>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4315,10 +4315,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>22.8</v>
+        <v>21.8</v>
       </c>
       <c r="C89" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -4333,12 +4333,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4359,10 +4359,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>20.3</v>
+        <v>18.9</v>
       </c>
       <c r="C90" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -4377,12 +4377,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva fraca</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4403,10 +4403,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>22.1</v>
+        <v>21.3</v>
       </c>
       <c r="C91" t="n">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -4421,12 +4421,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Sem chuva</t>
+          <t>Chuva moderada</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Atualização Automática: Dados IPMA
</commit_message>
<xml_diff>
--- a/Painel_Mestre_IPMA.xlsx
+++ b/Painel_Mestre_IPMA.xlsx
@@ -490,13 +490,13 @@
         <v>19.6</v>
       </c>
       <c r="C2" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
       <c r="D2" t="n">
-        <v>0.998</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7070000000000001</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -531,16 +531,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="C3" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.96</v>
+        <v>0.966</v>
       </c>
       <c r="E3" t="n">
-        <v>0.743</v>
+        <v>0.7390000000000001</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -575,16 +575,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="C4" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>0.968</v>
+        <v>0.95</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6459999999999999</v>
+        <v>0.628</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -619,16 +619,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="C5" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9690000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.632</v>
+        <v>0.627</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -663,16 +663,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="D6" t="n">
-        <v>0.992</v>
+        <v>0.9890000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.647</v>
+        <v>0.674</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -710,13 +710,13 @@
         <v>19.7</v>
       </c>
       <c r="C7" t="n">
-        <v>12.2</v>
+        <v>12</v>
       </c>
       <c r="D7" t="n">
-        <v>0.998</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7090000000000001</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -751,16 +751,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="C8" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.642</v>
+        <v>0.6609999999999999</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -795,20 +795,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20.8</v>
+        <v>20.9</v>
       </c>
       <c r="C9" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="D9" t="n">
-        <v>0.971</v>
+        <v>0.9590000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>0.645</v>
+        <v>0.6709999999999999</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="C10" t="n">
         <v>11.4</v>
       </c>
       <c r="D10" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>0.675</v>
+        <v>0.731</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -883,20 +883,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="C11" t="n">
-        <v>10.1</v>
+        <v>10.3</v>
       </c>
       <c r="D11" t="n">
-        <v>0.973</v>
+        <v>0.9790000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.701</v>
+        <v>0.716</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -927,16 +927,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20.7</v>
+        <v>21.4</v>
       </c>
       <c r="C12" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9940000000000001</v>
+        <v>0.993</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6509999999999999</v>
+        <v>0.628</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -974,13 +974,13 @@
         <v>18.4</v>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.996</v>
+        <v>0.985</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7559999999999999</v>
+        <v>0.7340000000000001</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1015,16 +1015,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19.9</v>
+        <v>20.9</v>
       </c>
       <c r="C14" t="n">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
       <c r="D14" t="n">
-        <v>0.953</v>
+        <v>0.9840000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>0.659</v>
+        <v>0.649</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1059,16 +1059,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="C15" t="n">
-        <v>10.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.946</v>
+        <v>0.973</v>
       </c>
       <c r="E15" t="n">
-        <v>0.636</v>
+        <v>0.619</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="C16" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9840000000000001</v>
+        <v>0.9890000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>0.674</v>
+        <v>0.664</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1147,16 +1147,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20.8</v>
+        <v>21.5</v>
       </c>
       <c r="C17" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D17" t="n">
         <v>0.993</v>
       </c>
       <c r="E17" t="n">
-        <v>0.653</v>
+        <v>0.629</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="C18" t="n">
         <v>9.6</v>
@@ -1200,7 +1200,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0.642</v>
+        <v>0.647</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1235,16 +1235,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="C19" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>0.998</v>
+        <v>0.995</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6659999999999999</v>
+        <v>0.649</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1279,16 +1279,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7390000000000001</v>
+        <v>0.716</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1323,16 +1323,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="D21" t="n">
-        <v>0.996</v>
+        <v>0.997</v>
       </c>
       <c r="E21" t="n">
-        <v>0.711</v>
+        <v>0.6859999999999999</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1370,13 +1370,13 @@
         <v>19.2</v>
       </c>
       <c r="C22" t="n">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>0.9840000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6659999999999999</v>
+        <v>0.708</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1411,16 +1411,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="C23" t="n">
-        <v>10.2</v>
+        <v>11.5</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
       <c r="E23" t="n">
-        <v>0.787</v>
+        <v>0.7909999999999999</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1455,16 +1455,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>19.1</v>
+        <v>17.8</v>
       </c>
       <c r="C24" t="n">
-        <v>9.5</v>
+        <v>10.3</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>0.997</v>
       </c>
       <c r="E24" t="n">
-        <v>0.644</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1499,16 +1499,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>20.3</v>
+        <v>19.2</v>
       </c>
       <c r="C25" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9670000000000001</v>
+        <v>0.977</v>
       </c>
       <c r="E25" t="n">
-        <v>0.629</v>
+        <v>0.7070000000000001</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Chuva Moderada</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1543,16 +1543,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>16.6</v>
+        <v>16.8</v>
       </c>
       <c r="C26" t="n">
-        <v>7.7</v>
+        <v>8.9</v>
       </c>
       <c r="D26" t="n">
-        <v>0.993</v>
+        <v>0.973</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.715</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Chuva Moderada</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1590,13 +1590,13 @@
         <v>19.3</v>
       </c>
       <c r="C27" t="n">
-        <v>9.4</v>
+        <v>10.2</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0.9840000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6659999999999999</v>
+        <v>0.7090000000000001</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1631,16 +1631,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="C28" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7240000000000001</v>
+        <v>0.7509999999999999</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1675,16 +1675,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>19.7</v>
+        <v>18.9</v>
       </c>
       <c r="C29" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0.9890000000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>0.672</v>
+        <v>0.73</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Chuva Moderada</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1719,16 +1719,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>16.6</v>
+        <v>17.3</v>
       </c>
       <c r="C30" t="n">
-        <v>8.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D30" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7879999999999999</v>
+        <v>0.784</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1763,16 +1763,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>19.2</v>
+        <v>18.7</v>
       </c>
       <c r="C31" t="n">
-        <v>8.4</v>
+        <v>8.9</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0.997</v>
       </c>
       <c r="E31" t="n">
-        <v>0.698</v>
+        <v>0.75</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Chuva Moderada</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1807,16 +1807,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>17.8</v>
+        <v>18.8</v>
       </c>
       <c r="C32" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D32" t="n">
-        <v>0.987</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>0.726</v>
+        <v>0.644</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1851,16 +1851,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="C33" t="n">
-        <v>10.6</v>
+        <v>11.7</v>
       </c>
       <c r="D33" t="n">
-        <v>0.98</v>
+        <v>0.9490000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>0.73</v>
+        <v>0.718</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1895,16 +1895,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>16.6</v>
+        <v>17.8</v>
       </c>
       <c r="C34" t="n">
-        <v>8.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="D34" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>0.795</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1939,16 +1939,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>19.8</v>
       </c>
       <c r="C35" t="n">
-        <v>10.1</v>
+        <v>11.1</v>
       </c>
       <c r="D35" t="n">
-        <v>0.929</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>0.721</v>
+        <v>0.611</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1983,16 +1983,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="C36" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D36" t="n">
-        <v>0.987</v>
+        <v>0.993</v>
       </c>
       <c r="E36" t="n">
-        <v>0.721</v>
+        <v>0.653</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2027,16 +2027,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>17.9</v>
+        <v>18.9</v>
       </c>
       <c r="C37" t="n">
-        <v>9.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="D37" t="n">
-        <v>0.987</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>0.731</v>
+        <v>0.649</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2071,16 +2071,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>18.7</v>
+        <v>18.5</v>
       </c>
       <c r="C38" t="n">
-        <v>8.4</v>
+        <v>9</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>0.7120000000000001</v>
+        <v>0.624</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Chuva Moderada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2115,16 +2115,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="C39" t="n">
-        <v>9.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>0.703</v>
+        <v>0.653</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2159,20 +2159,20 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>17.2</v>
+        <v>17</v>
       </c>
       <c r="C40" t="n">
-        <v>9</v>
+        <v>10.3</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>0.758</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2203,16 +2203,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>18.2</v>
+        <v>18.9</v>
       </c>
       <c r="C41" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>0.6920000000000001</v>
+        <v>0.649</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2247,16 +2247,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="C42" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D42" t="n">
-        <v>0.9620000000000001</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>0.597</v>
+        <v>0.573</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2291,16 +2291,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="C43" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="D43" t="n">
-        <v>0.9109999999999999</v>
+        <v>0.9329999999999999</v>
       </c>
       <c r="E43" t="n">
-        <v>0.631</v>
+        <v>0.644</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2335,16 +2335,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>16.9</v>
+        <v>16.7</v>
       </c>
       <c r="C44" t="n">
-        <v>8.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D44" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>0.657</v>
+        <v>0.6559999999999999</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2379,16 +2379,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="C45" t="n">
-        <v>8.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="D45" t="n">
-        <v>0.903</v>
+        <v>0.98</v>
       </c>
       <c r="E45" t="n">
-        <v>0.599</v>
+        <v>0.589</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2397,12 +2397,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2423,25 +2423,25 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>15.5</v>
+        <v>15.1</v>
       </c>
       <c r="C46" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="D46" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>0.614</v>
+        <v>0.62</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2467,16 +2467,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>17.9</v>
+        <v>17.7</v>
       </c>
       <c r="C47" t="n">
-        <v>8.1</v>
+        <v>8.5</v>
       </c>
       <c r="D47" t="n">
-        <v>0.963</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>0.602</v>
+        <v>0.5770000000000001</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2511,16 +2511,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="C48" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>0.607</v>
+        <v>0.5770000000000001</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2555,16 +2555,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18.2</v>
+        <v>17.7</v>
       </c>
       <c r="C49" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="D49" t="n">
-        <v>0.973</v>
+        <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>0.625</v>
+        <v>0.604</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2599,16 +2599,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16.2</v>
+        <v>16.4</v>
       </c>
       <c r="C50" t="n">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="D50" t="n">
-        <v>0.9840000000000001</v>
+        <v>0.98</v>
       </c>
       <c r="E50" t="n">
-        <v>0.628</v>
+        <v>0.627</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2643,16 +2643,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17.9</v>
+        <v>17.7</v>
       </c>
       <c r="C51" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>0.62</v>
+        <v>0.585</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2687,13 +2687,17 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>19.7</v>
+        <v>20.4</v>
       </c>
       <c r="C52" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
+        <v>7.2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.9540000000000001</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.482</v>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2701,7 +2705,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2727,13 +2731,17 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="C53" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+        <v>9.9</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.9059999999999999</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.6659999999999999</v>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>Moderado</t>
@@ -2741,7 +2749,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2767,13 +2775,17 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="C54" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
+        <v>7.3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.532</v>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2781,12 +2793,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2807,13 +2819,17 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>20.1</v>
+        <v>20.4</v>
       </c>
       <c r="C55" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
+        <v>7.9</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.523</v>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2821,12 +2837,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2847,13 +2863,17 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>17.2</v>
+        <v>17.6</v>
       </c>
       <c r="C56" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+        <v>5.8</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.531</v>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2866,7 +2886,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2887,13 +2907,17 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="C57" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+        <v>7.4</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.488</v>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2901,7 +2925,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2927,13 +2951,17 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="C58" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
+        <v>6.7</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.501</v>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2941,7 +2969,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2967,13 +2995,17 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="C59" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
+        <v>7.3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.5479999999999999</v>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -2986,7 +3018,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3007,16 +3039,20 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17.8</v>
+        <v>18.4</v>
       </c>
       <c r="C60" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
+        <v>8.1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.608</v>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Fraco</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3047,13 +3083,17 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="C61" t="n">
-        <v>7</v>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
+        <v>6.5</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.573</v>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>Fraco</t>
@@ -3061,12 +3101,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3087,10 +3127,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
       <c r="C62" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
@@ -3101,7 +3141,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3127,10 +3167,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="C63" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
@@ -3167,10 +3207,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>20.5</v>
+        <v>21</v>
       </c>
       <c r="C64" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
@@ -3181,7 +3221,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3207,10 +3247,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>22.1</v>
+        <v>22.5</v>
       </c>
       <c r="C65" t="n">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
@@ -3221,7 +3261,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3247,10 +3287,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>19.3</v>
+        <v>19.9</v>
       </c>
       <c r="C66" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
@@ -3261,7 +3301,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3287,10 +3327,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>21.9</v>
+        <v>22.3</v>
       </c>
       <c r="C67" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
@@ -3301,7 +3341,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3327,10 +3367,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
       <c r="C68" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
@@ -3341,7 +3381,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3367,10 +3407,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>21.9</v>
+        <v>22.2</v>
       </c>
       <c r="C69" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
@@ -3407,21 +3447,21 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>19.9</v>
+        <v>20.6</v>
       </c>
       <c r="C70" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fraco</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3447,10 +3487,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="C71" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
@@ -3487,10 +3527,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>21.9</v>
+        <v>23.5</v>
       </c>
       <c r="C72" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
@@ -3527,10 +3567,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>19.5</v>
+        <v>19.8</v>
       </c>
       <c r="C73" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
@@ -3541,7 +3581,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3567,10 +3607,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>21.1</v>
+        <v>22.6</v>
       </c>
       <c r="C74" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
@@ -3586,7 +3626,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3607,10 +3647,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>22.4</v>
+        <v>23.9</v>
       </c>
       <c r="C75" t="n">
-        <v>8.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
@@ -3626,7 +3666,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3647,10 +3687,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>19.8</v>
+        <v>21.4</v>
       </c>
       <c r="C76" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
@@ -3666,7 +3706,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3687,10 +3727,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>22</v>
+        <v>23.6</v>
       </c>
       <c r="C77" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr"/>
@@ -3727,10 +3767,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>22.1</v>
+        <v>23.5</v>
       </c>
       <c r="C78" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
@@ -3767,7 +3807,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>22.3</v>
+        <v>23.8</v>
       </c>
       <c r="C79" t="n">
         <v>7.9</v>
@@ -3807,10 +3847,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>20</v>
+        <v>21.3</v>
       </c>
       <c r="C80" t="n">
-        <v>8.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
@@ -3821,7 +3861,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NW</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3847,10 +3887,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>22</v>
+        <v>23.3</v>
       </c>
       <c r="C81" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
@@ -3861,7 +3901,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3887,7 +3927,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>21.1</v>
+        <v>21.5</v>
       </c>
       <c r="C82" t="n">
         <v>9.5</v>
@@ -3901,12 +3941,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -3927,10 +3967,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>18.7</v>
+        <v>18.3</v>
       </c>
       <c r="C83" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
@@ -3941,12 +3981,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -3967,10 +4007,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="C84" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
@@ -3981,12 +4021,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4010,7 +4050,7 @@
         <v>22</v>
       </c>
       <c r="C85" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
@@ -4021,12 +4061,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4047,10 +4087,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="C86" t="n">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr"/>
@@ -4061,7 +4101,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4087,10 +4127,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>21.2</v>
+        <v>21.6</v>
       </c>
       <c r="C87" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
@@ -4101,12 +4141,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4127,10 +4167,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="C88" t="n">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr"/>
@@ -4141,12 +4181,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4167,10 +4207,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
       <c r="C89" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr"/>
@@ -4181,12 +4221,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Chuva Fraca</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4207,10 +4247,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="C90" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
@@ -4221,12 +4261,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Chuva Fraca</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4247,10 +4287,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>21.3</v>
+        <v>21.1</v>
       </c>
       <c r="C91" t="n">
-        <v>8.1</v>
+        <v>8.4</v>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
@@ -4261,12 +4301,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Chuva Moderada</t>
+          <t>Sem Chuva</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">

</xml_diff>